<commit_message>
Update sample sales data for portfolio screenshots
</commit_message>
<xml_diff>
--- a/data/input/sample_sales_2026_04.xlsx
+++ b/data/input/sample_sales_2026_04.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="売上データ" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'売上データ'!$A$1:$F$23</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +27,21 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +56,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,33 +427,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>quantity</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>unit_price</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>日付</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>商品名</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>カテゴリ</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>単価</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>金額</t>
         </is>
       </c>
     </row>
@@ -451,68 +478,572 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>りんご</t>
+          <t>オーガニックコーヒー</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>果物</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E2" t="n">
-        <v>120</v>
+          <t>飲料</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>780</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>9360</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>みかん</t>
+          <t>米粉クッキー</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>果物</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>8</v>
-      </c>
-      <c r="E3" t="n">
-        <v>100</v>
+          <t>食品</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>5250</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ハーブティー</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>飲料</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>680</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>6120</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>2026-04-03</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ノート</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>エコバッグ</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>雑貨</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>8400</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ビジネスノート</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>文具</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D6" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>480</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>6720</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ジェルボールペン</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>文具</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>3960</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ハンドソープ</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>日用品</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>620</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>6200</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>キッチンタオル</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>日用品</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>540</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>4860</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>季節限定ギフトセット</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ギフト</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E4" t="n">
-        <v>200</v>
+      <c r="E10" s="2" t="n">
+        <v>2800</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>オーガニックコーヒー</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>飲料</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>780</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>10920</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>米粉クッキー</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>食品</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>4550</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ハーブティー</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>飲料</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>680</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>7480</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>エコバッグ</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>雑貨</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ビジネスノート</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>文具</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>480</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>5760</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ハンドソープ</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>日用品</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>620</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>5580</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>季節限定ギフトセット</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ギフト</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>2800</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>16800</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>キッチンタオル</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>日用品</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>540</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>5940</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>オーガニックコーヒー</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>飲料</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>780</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>10140</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ジェルボールペン</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>文具</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>米粉クッキー</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>食品</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>5600</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ステンレスボトル</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>雑貨</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ステンレスボトル</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>雑貨</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>7200</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>